<commit_message>
Sync GRC_Master.xlsx evidence tracker with CSV
</commit_message>
<xml_diff>
--- a/artifacts/11_GRC_Tooling/GRC_Master.xlsx
+++ b/artifacts/11_GRC_Tooling/GRC_Master.xlsx
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -733,6 +733,454 @@
           <t>Notes</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SOC2-AC-01 / SDG-AC-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CT-01 TOTP MFA workpaper + screenshots</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Badr Karim</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Screenshot + notes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Per release</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Redact OTP codes and never show otp_secret</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SOC2-AC-02 / SDG-AC-02</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CT-02 RBAC workpaper + deny proofs</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Badr Karim</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Screenshot + notes</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>E-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SOC2-LG-01 / SDG-LG-01</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>audit_logs export (sanitized columns)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Badr Karim</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DB export (CSV)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>artifacts/14_Evidence/2026-02/SOC2_SEC_CT-03_AuditLogs_Export_2026-02-28.csv</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Use export script; redact sensitive IPs if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>E-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SOC2-LG-01 / SDG-LG-02</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>query_runs export (sanitized columns)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Badr Karim</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DB export (CSV)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>artifacts/14_Evidence/2026-02/SOC2_SEC_CT-03_QueryRuns_Sanitized_2026-02-28.csv</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Do not export params/tracebacks in public evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SDG-IN-01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>integrity_snapshots export (limited fields)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Badr Karim</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DB export (CSV)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>artifacts/14_Evidence/2026-02/SDG_IN_IntegritySnapshots_Export_2026-02-28.csv</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>E-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SDG-AC-03</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Quarterly access review record</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Badr Karim</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Record + RBAC export</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>E-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SDG-LG-03</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Weekly log review checklist completion</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Badr Karim</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Checklist + notes</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>E-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SDG-SDLC-01</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Hygiene check pass output</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Badr Karim</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Command output capture</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Per release</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Store as PDF or text evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>E-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SDG-CH-01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Change review checklist</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Badr Karim</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Checklist completion</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Per release</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>E-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SDG-TPRM-01</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Vendor review note + tracker update</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Badr Karim</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Note + CSV update</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>E-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SDG-DP-01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Data inventory/classification/retention/DPIA pack</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Badr Karim</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Document pack</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: clear pending states and update evidence links in workpapers and trackers
</commit_message>
<xml_diff>
--- a/artifacts/11_GRC_Tooling/GRC_Master.xlsx
+++ b/artifacts/11_GRC_Tooling/GRC_Master.xlsx
@@ -765,9 +765,6 @@
           <t>Per release</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Redact OTP codes and never show otp_secret</t>
@@ -805,10 +802,6 @@
           <t>Monthly</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -960,7 +953,6 @@
           <t>artifacts/14_Evidence/2026-02/SDG_IN_IntegritySnapshots_Export_2026-02-28.csv</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -993,10 +985,6 @@
           <t>Quarterly</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1029,10 +1017,6 @@
           <t>Weekly</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1065,9 +1049,6 @@
           <t>Per release</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>Store as PDF or text evidence</t>
@@ -1105,10 +1086,6 @@
           <t>Per release</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1141,10 +1118,6 @@
           <t>Quarterly</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1177,10 +1150,6 @@
           <t>Annual</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sync GRC_Master.xlsx after evidence cadence fix
</commit_message>
<xml_diff>
--- a/artifacts/11_GRC_Tooling/GRC_Master.xlsx
+++ b/artifacts/11_GRC_Tooling/GRC_Master.xlsx
@@ -765,6 +765,9 @@
           <t>Per release</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Redact OTP codes and never show otp_secret</t>
@@ -802,6 +805,10 @@
           <t>Monthly</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -841,7 +848,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -893,7 +900,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -945,7 +952,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -953,6 +960,7 @@
           <t>artifacts/14_Evidence/2026-02/SDG_IN_IntegritySnapshots_Export_2026-02-28.csv</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -985,6 +993,10 @@
           <t>Quarterly</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1017,6 +1029,10 @@
           <t>Weekly</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1049,6 +1065,9 @@
           <t>Per release</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>Store as PDF or text evidence</t>
@@ -1086,6 +1105,10 @@
           <t>Per release</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1118,6 +1141,10 @@
           <t>Quarterly</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1150,6 +1177,10 @@
           <t>Annual</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>